<commit_message>
Add dual-sheet Excel export: לשלישות + פנימי
- scheduler.py: add allow_double_shift, no_double_shift_weekday, ignore_constraints params
- excel_export.py: refactor to write two sheets via _write_schedule_sheet helper
- week_29_03.py: generate two schedules and export to single workbook

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/משמרות_29.3-4.4.xlsx
+++ b/משמרות_29.3-4.4.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="משמרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="לשלישות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פנימי" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,9 +39,8 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -48,12 +48,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FFFFFF"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -90,8 +90,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF00FF"/>
-        <bgColor rgb="00FF00FF"/>
+        <fgColor rgb="0000B050"/>
+        <bgColor rgb="0000B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
@@ -102,20 +114,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-        <bgColor rgb="00FFC000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0000B050"/>
-        <bgColor rgb="0000B050"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FF00FF"/>
+        <bgColor rgb="00FF00FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -151,13 +151,13 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -166,23 +166,25 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -556,17 +558,17 @@
   <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="55" customHeight="1">
+    <row r="1" ht="52" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>תאריך
@@ -620,170 +622,167 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="50" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>משמרת
-בוקר
+          <t>בוקר
 8:00-16:00</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>ערב
+14:00-22:00</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>יהב</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
     </row>
-    <row r="3" ht="50" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>משמרת
-צהריים
-ערב
-14:00-22:00</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>משה</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>משה</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="50" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>לילה
 20:00-9:00</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>אורי</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>עומר</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>אורי</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>מקרא צבעים:</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
+          <t>מקרא:</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>עומרי</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>אורי</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>יהב</t>
         </is>
@@ -807,22 +806,303 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
+          <t>עומר: 6</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>עומרי: 5</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>אורי: 6</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>יהב: 1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="52" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>תאריך
+יום</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>29.03
+ראשון</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>30.03
+שני</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>31.03
+שלישי</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>01.04
+רביעי
+🔴 ערב פסח</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>02.04
+חמישי
+🔴 פסח</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>03.04
+שישי
+🔴 חול המועד פסח</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>04.04
+שבת
+🔴 חול המועד פסח</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>בוקר
+8:00-16:00</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>ערב
+14:00-22:00</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>יהב</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>לילה
+20:00-9:00</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>מקרא:</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>יהב</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>סה״כ נקודות:</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>ניר: 6</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>משה: 5</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
           <t>עומר: 5</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>עומרי: 5</t>
+          <t>עומרי: 6</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>אורי: 6</t>
+          <t>אורי: 5</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>יהב: 2</t>
+          <t>יהב: 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add fixed assignments, excluded employees, partial-week support
Engine: support for pre-assigned shifts, employee start dates,
and excluded employees. External sheet derived from internal
with double-shift redistribution and overrides.

Week 29.3-4.4: יהב out, אורי→צרפתי, אורי הלוי joins Wed (eve+night).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/משמרות_29.3-4.4.xlsx
+++ b/משמרות_29.3-4.4.xlsx
@@ -39,11 +39,11 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -90,20 +90,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000B050"/>
-        <bgColor rgb="0000B050"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
         <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-        <bgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
@@ -116,6 +104,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FF00FF"/>
         <bgColor rgb="00FF00FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B050"/>
+        <bgColor rgb="0000B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
@@ -160,7 +160,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -172,22 +172,22 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -631,37 +631,37 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
           <t>עומרי</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>עומרי</t>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>משה</t>
         </is>
       </c>
     </row>
@@ -672,39 +672,39 @@
 14:00-22:00</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>עומרי</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>משה</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>משה</t>
         </is>
       </c>
     </row>
@@ -717,37 +717,37 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
           <t>עומר</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>משה</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>יהב</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
           <t>ניר</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -772,7 +772,7 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>עומרי</t>
         </is>
@@ -796,7 +796,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ניר: 5</t>
+          <t>ניר: 6</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>עומר: 6</t>
+          <t>עומר: 5</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>אורי: 6</t>
+          <t>אורי: 5</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>יהב: 1</t>
+          <t>יהב: 2</t>
         </is>
       </c>
     </row>
@@ -910,37 +910,37 @@
 8:00-16:00</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
@@ -953,39 +953,39 @@
 14:00-22:00</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>אורי</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>משה</t>
         </is>
       </c>
     </row>
@@ -996,39 +996,39 @@
 20:00-9:00</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>אורי</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>עומרי</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>עומרי</t>
+          <t>אורי</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>עומרי</t>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>יהב</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>משה</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
           <t>ניר</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -1053,7 +1053,7 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>עומרי</t>
         </is>
@@ -1077,12 +1077,12 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ניר: 6</t>
+          <t>ניר: 5</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>משה: 5</t>
+          <t>משה: 6</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>עומרי: 6</t>
+          <t>עומרי: 5</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>יהב: 1</t>
+          <t>יהב: 2</t>
         </is>
       </c>
     </row>

</xml_diff>